<commit_message>
Update UBWC register docs and manuals
</commit_message>
<xml_diff>
--- a/docs/ubwc_dec_reg_table.xlsx
+++ b/docs/ubwc_dec_reg_table.xlsx
@@ -66,7 +66,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I59"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -165,12 +165,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>IP version</t>
+          <t>IP version register.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Returns fixed value 32'h0001_0000</t>
+          <t>Read once after reset to confirm software/RTL compatibility.</t>
         </is>
       </c>
     </row>
@@ -212,12 +212,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>RTL date</t>
+          <t>RTL date register.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Returns fixed value 32'h2026_0403</t>
+          <t>Read once after reset to confirm software/RTL compatibility.</t>
         </is>
       </c>
     </row>
@@ -259,12 +259,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Level-1 bank swizzle enable</t>
+          <t>Level-1 bank swizzle enable; stored for readback.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Software default writes 0. Combined bank swizzle default [2:0]=3'b110.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -306,12 +306,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Level-2 bank swizzle enable</t>
+          <t>Level-2 bank swizzle enable; latched to AXI domain at frame start.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Software default writes 1. Combined bank swizzle default [2:0]=3'b110.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -353,12 +353,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Level-3 bank swizzle enable</t>
+          <t>Level-3 bank swizzle enable; latched to AXI domain at frame start.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Software default writes 1. Combined bank swizzle default [2:0]=3'b110.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -400,12 +400,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Highest bank bit configuration</t>
+          <t>Highest bank bit.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t/>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -447,12 +447,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Bank spread enable</t>
+          <t>Bank spread enable.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Software default writes 1.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -484,22 +484,22 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>tile_cfg_is_lossy_rgba_2_1_format</t>
+          <t>tile_cfg_4line_format</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>RGBA 2:1 lossy format select</t>
+          <t>4-line tile format; stored for readback.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Only applies to RGBA8888 metadata/tile address path. 0=normal RGBA/lossless layout, 1=RGBA8888 lossy 2:1 layout. When 1, decoder halves the effective tile_y for address calculation, adds a 128-byte offset for odd tile_y, disables bank spread for this path, and treats 256-byte metadata payload as 128 bytes.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -511,12 +511,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>0x000c</t>
+          <t>0x0008</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>APB_ADDR_TILE_CFG1</t>
+          <t>APB_ADDR_TILE_CFG0</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -531,22 +531,22 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>11:0</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>tile_cfg_pitch</t>
+          <t>tile_cfg_is_lossy_rgba_2_1_format</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Tile pitch configuration</t>
+          <t>RGBA8888 lossy 2:1 layout select.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Tile surface pitch in 16-byte units. Program tile_cfg_pitch=align_up(width*bpp, tile_w*4*bpp)/16. bpp: RGBA8888/RGBA1010102=4, YUV420_8=1, YUV420_10=2. tile_w: RGBA=16, YUV=32. RTL uses tile_cfg_pitch&lt;&lt;4 as byte pitch. Example NV12 1996x1074: align_up(1996*1,32*4*1)=2048 bytes, tile_cfg_pitch=2048/16=128.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -558,12 +558,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>0x0010</t>
+          <t>0x000c</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>APB_ADDR_TILE_CFG2</t>
+          <t>APB_ADDR_TILE_CFG1</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -578,22 +578,22 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>11:0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>tile_cfg_ci_input_type</t>
+          <t>tile_cfg_pitch</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>CI input type</t>
+          <t>Tile pitch in 16-byte units.</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>0=linear data, 1=tiled data. Software default writes 1.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -625,22 +625,22 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>tile_cfg_ci_lossy</t>
+          <t>tile_cfg_ci_input_type</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>CI lossy enable</t>
+          <t>CI input type. Software should write 1 for tiled CI.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Software writes 1 for lossy format and 0 for lossless format.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -672,22 +672,22 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>10:9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>tile_cfg_ci_alpha_mode</t>
+          <t>tile_cfg_ci_lossy</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>CI alpha mode configuration</t>
+          <t>CI lossy enable.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Reserved. Software should write 0.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -699,12 +699,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>0x0014</t>
+          <t>0x0010</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>APB_ADDR_VIVO_CFG</t>
+          <t>APB_ADDR_TILE_CFG2</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -714,27 +714,27 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>0x00000001</t>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10:9</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>vivo_ubwc_en</t>
+          <t>tile_cfg_ci_alpha_mode</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>ubwc_dec_vivo_top enable</t>
+          <t>CI alpha mode.</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Defaults to 1 after reset</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -766,22 +766,22 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>vivo_sreset</t>
+          <t>vivo_ubwc_en</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>VIVO submodule soft reset</t>
+          <t>VIVO UBWC path enable.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Can be used to independently clear VIVO internal state</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -793,12 +793,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>0x0018</t>
+          <t>0x0014</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>APB_ADDR_OTF_CFG0</t>
+          <t>APB_ADDR_VIVO_CFG</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -813,22 +813,22 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>15:0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>otf_cfg_img_width</t>
+          <t>vivo_sreset</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Valid output image width in pixels</t>
+          <t>VIVO soft reset.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Program active image width in pixels. Used to limit line unpacking: RGBA words=ceil(width/4), YUV420_8/NV12 words=ceil(width/16), YUV420_10/P010 words=ceil(width/8).</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -860,22 +860,22 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>15:0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>otf_cfg_format</t>
+          <t>otf_cfg_img_width</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Output OTF format</t>
+          <t>Valid output image width in pixels.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Frame-level output format. Codes: 0=RGBA8888, 1=RGBA1010102, 2=YUV420_8/NV12, 3=YUV420_10/P010. Also drives meta_base_format.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -887,12 +887,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>0x001c</t>
+          <t>0x0018</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>APB_ADDR_OTF_CFG1</t>
+          <t>APB_ADDR_OTF_CFG0</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -907,22 +907,22 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>15:0</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>otf_cfg_h_total</t>
+          <t>otf_cfg_format</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>OTF H_TOTAL</t>
+          <t>Output OTF format; also drives meta_base_format.</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Horizontal total in pixels. RTL converts to OTF beats with ceil(h_total/4). Must cover h_sync + h_bp + h_act.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -954,22 +954,22 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>31:16</t>
+          <t>15:0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>otf_cfg_h_sync</t>
+          <t>otf_cfg_h_total</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>OTF H_SYNC</t>
+          <t>Horizontal total.</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Horizontal sync width in pixels. RTL converts to OTF beats with ceil(h_sync/4).</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -981,12 +981,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>0x0020</t>
+          <t>0x001c</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>APB_ADDR_OTF_CFG2</t>
+          <t>APB_ADDR_OTF_CFG1</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1001,22 +1001,22 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>15:0</t>
+          <t>31:16</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>otf_cfg_h_bp</t>
+          <t>otf_cfg_h_sync</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>OTF H_BP</t>
+          <t>Horizontal sync width.</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Horizontal back porch in pixels. RTL converts to OTF beats with ceil(h_bp/4). Active window starts after h_sync + h_bp.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -1048,22 +1048,22 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>31:16</t>
+          <t>15:0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>otf_cfg_h_act</t>
+          <t>otf_cfg_h_bp</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>OTF H_ACT</t>
+          <t>Horizontal back porch.</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Horizontal active width in pixels. Usually program the visible output width; should match otf_cfg_img_width unless blanking/active width is intentionally different.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1075,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>0x0024</t>
+          <t>0x0020</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>APB_ADDR_OTF_CFG3</t>
+          <t>APB_ADDR_OTF_CFG2</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1095,22 +1095,22 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>15:0</t>
+          <t>31:16</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>otf_cfg_v_total</t>
+          <t>otf_cfg_h_act</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>OTF V_TOTAL</t>
+          <t>Horizontal active width.</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Vertical total in lines. Must cover v_sync + v_bp + v_act.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -1142,22 +1142,22 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>31:16</t>
+          <t>15:0</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>otf_cfg_v_sync</t>
+          <t>otf_cfg_v_total</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>OTF V_SYNC</t>
+          <t>Vertical total.</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Vertical sync width in lines.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -1169,12 +1169,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>0x0028</t>
+          <t>0x0024</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>APB_ADDR_OTF_CFG4</t>
+          <t>APB_ADDR_OTF_CFG3</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1189,22 +1189,22 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>15:0</t>
+          <t>31:16</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>otf_cfg_v_bp</t>
+          <t>otf_cfg_v_sync</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>OTF V_BP</t>
+          <t>Vertical sync width.</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Vertical back porch in lines. Active window starts after v_sync + v_bp.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -1236,22 +1236,22 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>31:16</t>
+          <t>15:0</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>otf_cfg_v_act</t>
+          <t>otf_cfg_v_bp</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>OTF V_ACT</t>
+          <t>Vertical back porch.</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Vertical active height in lines. Program the visible output height.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -1263,12 +1263,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>0x002c</t>
+          <t>0x0028</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>APB_ADDR_META_CFG0</t>
+          <t>APB_ADDR_OTF_CFG4</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1283,22 +1283,22 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>15:0</t>
+          <t>31:16</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>meta_tile_x_numbers</t>
+          <t>otf_cfg_v_act</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Y/RGBA metadata tile columns</t>
+          <t>Vertical active height.</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>YUV420 UV metadata columns are derived by format. ceil(a/b) means round up division.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -1330,22 +1330,22 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>31:16</t>
+          <t>15:0</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>meta_tile_y_numbers</t>
+          <t>meta_tile_x_numbers</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Y/RGBA metadata tile rows</t>
+          <t>Y/RGBA metadata tile columns; YUV420 UV columns are derived by format.</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>For YUV420, UV metadata rows are derived internally as round_up(meta_tile_y_numbers/2).</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -1357,12 +1357,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>0x0030</t>
+          <t>0x002c</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>REG_META_BASE_Y_LO</t>
+          <t>APB_ADDR_META_CFG0</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1377,22 +1377,22 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>31:0</t>
+          <t>31:16</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>meta_base_addr_rgba_y[31:0]</t>
+          <t>meta_tile_y_numbers</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Low 32 bits of the RGBA or Y metadata base address</t>
+          <t>Y/RGBA metadata tile rows; YUV420 UV rows are derived internally.</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>For contiguous UBWC buffer, program Y/RGBA metadata start address. Metadata size formula: meta_pitch=align_up(ceil(plane_width/tile_w),64); meta_size=align_up(meta_pitch*align_up(ceil(plane_height/tile_h),16),4KB). Example NV12 1996x1074 base=0xA00000: Y meta_base=0xA00000, Y meta_pitch=64, Y meta_size=0x3000.</t>
+          <t>Configure when image format, size, layout, or timing changes. Reuse when only frame buffer addresses change.</t>
         </is>
       </c>
     </row>
@@ -1404,12 +1404,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>0x0034</t>
+          <t>0x0030</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>REG_META_BASE_Y_HI</t>
+          <t>REG_META_BASE_Y_LO</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1429,17 +1429,17 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>meta_base_addr_rgba_y[63:32]</t>
+          <t>meta_base_addr_rgba_y[31:0]</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>High 32 bits of the RGBA or Y metadata base address</t>
+          <t>RGBA/Y metadata base address low word.</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Write after REG_META_BASE_Y_LO to complete this 64-bit base address.</t>
+          <t>Per-frame configuration. Low/high words form one 64-bit base address.</t>
         </is>
       </c>
     </row>
@@ -1451,12 +1451,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>0x0038</t>
+          <t>0x0034</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>REG_TILE_BASE_Y_LO</t>
+          <t>REG_META_BASE_Y_HI</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1476,17 +1476,17 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>tile_base_addr_rgba_y[31:0]</t>
+          <t>meta_base_addr_rgba_y[63:32]</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Low 32 bits of the RGBA or Y compressed tile base address</t>
+          <t>RGBA/Y metadata base address high word.</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>For YUV formats, program Y pixel/tile data start. Example NV12 1996x1074: Y tile_base = Y_meta_base + Y_meta_size = 0xA00000 + 0x3000 = 0xA03000.</t>
+          <t>Per-frame configuration. Low/high words complete this base address.</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>0x003c</t>
+          <t>0x0038</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>REG_TILE_BASE_Y_HI</t>
+          <t>REG_TILE_BASE_Y_LO</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1523,17 +1523,17 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>tile_base_addr_rgba_y[63:32]</t>
+          <t>tile_base_addr_rgba_y[31:0]</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>High 32 bits of the RGBA or Y compressed tile base address</t>
+          <t>RGBA/Y compressed tile data base address low word.</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Write after REG_TILE_BASE_Y_LO to complete this 64-bit base address.</t>
+          <t>Per-frame configuration. Low/high words form one 64-bit base address.</t>
         </is>
       </c>
     </row>
@@ -1545,12 +1545,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>0x0040</t>
+          <t>0x003c</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>REG_META_BASE_UV_LO</t>
+          <t>REG_TILE_BASE_Y_HI</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1570,17 +1570,17 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>meta_base_addr_uv[31:0]</t>
+          <t>tile_base_addr_rgba_y[63:32]</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Low 32 bits of the UV metadata base address</t>
+          <t>RGBA/Y compressed tile data base address high word.</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>For YUV formats, program UV metadata start address. Example NV12 1996x1074 contiguous layout: meta_base_uv = tile_base_y + Y_pixel_size = 0xA03000 + 0x220000 = 0xC23000.</t>
+          <t>Per-frame configuration. Low/high words complete this base address.</t>
         </is>
       </c>
     </row>
@@ -1592,12 +1592,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>0x0044</t>
+          <t>0x0040</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>REG_META_BASE_UV_HI</t>
+          <t>REG_META_BASE_UV_LO</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1617,17 +1617,17 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>meta_base_addr_uv[63:32]</t>
+          <t>meta_base_addr_uv[31:0]</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>High 32 bits of the UV metadata base address</t>
+          <t>UV metadata base address low word.</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Write after REG_META_BASE_UV_LO to complete this 64-bit base address.</t>
+          <t>Per-frame configuration. Low/high words form one 64-bit base address.</t>
         </is>
       </c>
     </row>
@@ -1639,12 +1639,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>0x0048</t>
+          <t>0x0044</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>REG_TILE_BASE_UV_LO</t>
+          <t>REG_META_BASE_UV_HI</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1664,17 +1664,17 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>tile_base_addr_uv[31:0]</t>
+          <t>meta_base_addr_uv[63:32]</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Low 32 bits of the UV compressed tile base address</t>
+          <t>UV metadata base address high word.</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>For YUV formats, program UV pixel/tile data start. RGBA format does not use this address.</t>
+          <t>Per-frame configuration. Low/high words complete this base address.</t>
         </is>
       </c>
     </row>
@@ -1686,12 +1686,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>0x004c</t>
+          <t>0x0048</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>REG_TILE_BASE_UV_HI</t>
+          <t>REG_TILE_BASE_UV_LO</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1711,17 +1711,17 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>tile_base_addr_uv[63:32]</t>
+          <t>tile_base_addr_uv[31:0]</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>High 32 bits of the UV compressed tile base address</t>
+          <t>UV compressed tile data base address low word. RGBA format does not use this address.</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Write after REG_TILE_BASE_UV_LO to complete this 64-bit base address. RGBA format does not use this address.</t>
+          <t>Per-frame configuration. Low/high words form one 64-bit base address.</t>
         </is>
       </c>
     </row>
@@ -1733,42 +1733,42 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>0x0050</t>
+          <t>0x004c</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>APB_ADDR_STATUS0</t>
+          <t>REG_TILE_BASE_UV_HI</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>RO</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>31:0</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>frame_active</t>
+          <t>tile_base_addr_uv[63:32]</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Whether the current frame is active</t>
+          <t>UV compressed tile data base address high word. RGBA format does not use this address.</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Set to 1 after start; cleared to 0 when the current frame fully completes</t>
+          <t>Per-frame configuration. Low/high words complete this base address.</t>
         </is>
       </c>
     </row>
@@ -1800,22 +1800,22 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>meta_busy</t>
+          <t>frame_active</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Metadata read stage busy</t>
+          <t>Current frame active.</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t/>
+          <t>Read-only status or statistic information.</t>
         </is>
       </c>
     </row>
@@ -1847,22 +1847,22 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>tile_busy</t>
+          <t>meta_busy</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Tile read stage busy</t>
+          <t>Metadata stage busy.</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t/>
+          <t>Read during runtime.</t>
         </is>
       </c>
     </row>
@@ -1894,22 +1894,22 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>vivo_busy</t>
+          <t>tile_busy</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>ubwc_dec_vivo_top busy</t>
+          <t>Tile address/read stage busy.</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t/>
+          <t>Read during runtime.</t>
         </is>
       </c>
     </row>
@@ -1941,22 +1941,22 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>otf_busy</t>
+          <t>vivo_busy</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>tile_to_otf stage busy</t>
+          <t>VIVO stage busy.</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t/>
+          <t>Read during runtime.</t>
         </is>
       </c>
     </row>
@@ -1988,22 +1988,22 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>all_stage_idle</t>
+          <t>otf_busy</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>All current busy inputs are 0</t>
+          <t>Tile-to-OTF stage busy.</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>May be 1 before start and after completion</t>
+          <t>Read during runtime.</t>
         </is>
       </c>
     </row>
@@ -2035,22 +2035,22 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>frame_idle_done</t>
+          <t>all_stage_idle</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>No current busy and frame_active=0</t>
+          <t>No current busy stage.</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Recommended to combine with STATUS1[4] to judge frame completion</t>
+          <t>Read during runtime.</t>
         </is>
       </c>
     </row>
@@ -2062,12 +2062,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>0x0054</t>
+          <t>0x0050</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>APB_ADDR_STATUS1</t>
+          <t>APB_ADDR_STATUS0</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2075,29 +2075,29 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>0x00000000</t>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>meta_done</t>
+          <t>frame_idle_done</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Metadata stage completed</t>
+          <t>No busy stage and frame_active=0.</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Cleared when a new frame starts</t>
+          <t>Read during runtime.</t>
         </is>
       </c>
     </row>
@@ -2122,29 +2122,29 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>0x00000000</t>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4:0</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>tile_done</t>
+          <t>stage_done</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Tile stage completed</t>
+          <t>Done bitmap: bit0 meta, bit1 tile address, bit2 reserved, bit3 otf, bit4 frame.</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Cleared when a new frame starts</t>
+          <t>Read during runtime.</t>
         </is>
       </c>
     </row>
@@ -2169,29 +2169,29 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>0x00000000</t>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8:5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>reserved</t>
+          <t>stage_seen</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Reserved; reads 0</t>
+          <t>Stage-seen-busy bitmap for meta/tile/vivo/otf.</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>VIVO completion is not latched as a done condition</t>
+          <t>Read-only status or statistic information.</t>
         </is>
       </c>
     </row>
@@ -2203,12 +2203,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>0x0054</t>
+          <t>0x0058</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>APB_ADDR_STATUS1</t>
+          <t>APB_ADDR_STATUS2</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2216,29 +2216,29 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>0x00000000</t>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6:0</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>otf_done</t>
+          <t>vivo_idle_bits</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>OTF output stage completed</t>
+          <t>Raw VIVO idle bitmap.</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Cleared when a new frame starts</t>
+          <t>Read during runtime.</t>
         </is>
       </c>
     </row>
@@ -2250,12 +2250,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>0x0054</t>
+          <t>0x005c</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>APB_ADDR_STATUS1</t>
+          <t>APB_ADDR_STATUS3</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2263,29 +2263,29 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>0x00000000</t>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6:0</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>frame_done</t>
+          <t>vivo_error_bits</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Full-frame completion flag</t>
+          <t>Raw VIVO error bitmap.</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Most recommended software polling bit</t>
+          <t>Read during runtime.</t>
         </is>
       </c>
     </row>
@@ -2297,42 +2297,42 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>0x0054</t>
+          <t>0x0060</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>APB_ADDR_STATUS1</t>
+          <t>APB_ADDR_IRQ_CTRL</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>0x00000000</t>
+          <t>0x00000001</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>meta_seen_busy</t>
+          <t>irq_enable</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Metadata stage entered busy during this frame</t>
+          <t>Interrupt enable.</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Used to avoid falsely judging done before start</t>
+          <t>Configure after reset or when the interrupt policy changes.</t>
         </is>
       </c>
     </row>
@@ -2344,17 +2344,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>0x0054</t>
+          <t>0x0060</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>APB_ADDR_STATUS1</t>
+          <t>APB_ADDR_IRQ_CTRL</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>W1P</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -2364,22 +2364,22 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>tile_seen_busy</t>
+          <t>irq_clear</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Tile stage entered busy during this frame</t>
+          <t>Write 1 to clear latched correct/error interrupt status.</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Same as above</t>
+          <t>Write 1 after software handles the interrupt; readback is 0.</t>
         </is>
       </c>
     </row>
@@ -2391,12 +2391,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>0x0054</t>
+          <t>0x0060</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>APB_ADDR_STATUS1</t>
+          <t>APB_ADDR_IRQ_CTRL</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2404,29 +2404,29 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>0x00000000</t>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>vivo_seen_busy</t>
+          <t>irq_pending</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>VIVO stage entered busy during this frame</t>
+          <t>Any pending interrupt.</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Same as above</t>
+          <t>Read during runtime or after interrupt handling for status/debug.</t>
         </is>
       </c>
     </row>
@@ -2438,12 +2438,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>0x0054</t>
+          <t>0x0060</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>APB_ADDR_STATUS1</t>
+          <t>APB_ADDR_IRQ_CTRL</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2451,29 +2451,29 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>0x00000000</t>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>otf_seen_busy</t>
+          <t>irq_error_pending</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>OTF stage entered busy during this frame</t>
+          <t>Error interrupt pending.</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Same as above</t>
+          <t>Read during runtime or after interrupt handling for status/debug.</t>
         </is>
       </c>
     </row>
@@ -2485,12 +2485,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>0x0058</t>
+          <t>0x0060</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>APB_ADDR_STATUS2</t>
+          <t>APB_ADDR_IRQ_CTRL</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2505,22 +2505,22 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>6:0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>vivo_idle_bits</t>
+          <t>irq_correct_pending</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Raw ubwc_dec_vivo_top idle bitmap</t>
+          <t>Correct/frame interrupt pending.</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Passed through as o_idle[6:0] for software debug</t>
+          <t>Read during runtime or after interrupt handling for status/debug.</t>
         </is>
       </c>
     </row>
@@ -2532,42 +2532,42 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>0x005c</t>
+          <t>0x0060</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>APB_ADDR_STATUS3</t>
+          <t>APB_ADDR_IRQ_CTRL</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>RO</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+          <t>W1P</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>6:0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>vivo_error_bits</t>
+          <t>start</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Raw ubwc_dec_vivo_top error bitmap</t>
+          <t>Write 1 after one full input UBWC address group has been configured. Address writes only fill the pending address queues; start is a separate frame token.</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Passed through as o_error[6:0] for software debug</t>
+          <t>Write 1 after the per-frame address group is complete; readback is 0. Address writes do not start a frame by themselves.</t>
         </is>
       </c>
     </row>
@@ -2579,42 +2579,42 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>0x0060</t>
+          <t>0x0064</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>APB_ADDR_IRQ_CTRL</t>
+          <t>APB_ADDR_STATUS4</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>RW/W1P</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>0x00000001</t>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>irq_enable</t>
+          <t>irq_status</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>IRQ enable</t>
+          <t>Bit0 any IRQ, bit1 error IRQ, bit2 correct IRQ.</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Defaults to 1 after reset</t>
+          <t>Read during runtime or after interrupt handling for status/debug.</t>
         </is>
       </c>
     </row>
@@ -2626,42 +2626,42 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>0x0060</t>
+          <t>0x0068</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>APB_ADDR_IRQ_CTRL</t>
+          <t>APB_ADDR_STAT_META</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>W1P</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>0x00000001</t>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>31:0</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>irq_clear</t>
+          <t>stat_meta_tile_cnt</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>IRQ clear pulse</t>
+          <t>Metadata valid tile count for the current/last frame.</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Writing 1 generates an irq_clear pulse in the AXI clock domain; readback is 0</t>
+          <t>Read during runtime or after interrupt handling for status/debug.</t>
         </is>
       </c>
     </row>
@@ -2673,12 +2673,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>0x0060</t>
+          <t>0x006c</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>APB_ADDR_IRQ_CTRL</t>
+          <t>APB_ADDR_STAT_TILE</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2693,22 +2693,22 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>31:0</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>irq_pending</t>
+          <t>stat_tile_addr_cnt</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>IRQ pending status</t>
+          <t>Tile address generator valid tile count.</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Synchronized into PCLK domain</t>
+          <t>Read during runtime or after interrupt handling for status/debug.</t>
         </is>
       </c>
     </row>
@@ -2720,12 +2720,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>0x0060</t>
+          <t>0x0070</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>APB_ADDR_IRQ_CTRL</t>
+          <t>APB_ADDR_STAT_OTF_TILE</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2740,22 +2740,22 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>31:0</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>irq_error_pending</t>
+          <t>stat_otf_tile_cnt</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Error IRQ pending status</t>
+          <t>Tile-to-OTF accepted tile count.</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Synchronized into PCLK domain</t>
+          <t>Read during runtime or after interrupt handling for status/debug.</t>
         </is>
       </c>
     </row>
@@ -2767,12 +2767,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>0x0060</t>
+          <t>0x0074</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>APB_ADDR_IRQ_CTRL</t>
+          <t>APB_ADDR_STAT_OTF_LINE</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2787,22 +2787,22 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>31:0</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>irq_correct_pending</t>
+          <t>stat_otf_line_cnt</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Correct/frame IRQ pending status</t>
+          <t>OTF output line count.</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Synchronized into PCLK domain</t>
+          <t>Read during runtime or after interrupt handling for status/debug.</t>
         </is>
       </c>
     </row>
@@ -2814,12 +2814,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>0x0064</t>
+          <t>0x0078</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>APB_ADDR_STATUS4</t>
+          <t>APB_ADDR_STAT_OTF_DE</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2834,262 +2834,27 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>31:0</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>irq_status</t>
+          <t>stat_otf_de_cnt</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Bit0 any IRQ, bit1 error IRQ, bit2 correct IRQ</t>
+          <t>OTF output data-enable beat count.</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Synchronized into PCLK domain</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>ubwc_dec_apb_reg_blk</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>0x0068</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>APB_ADDR_STAT_META</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>RO</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>dynamic</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>31:0</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>stat_meta_tile_cnt</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>Metadata valid tile count</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>Current or last frame debug counter</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>ubwc_dec_apb_reg_blk</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>0x006c</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>APB_ADDR_STAT_TILE</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>RO</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>dynamic</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>31:0</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>stat_tile_addr_cnt</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>Tile address valid tile count</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>Current or last frame debug counter</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>ubwc_dec_apb_reg_blk</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>0x0070</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>APB_ADDR_STAT_OTF_TILE</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>RO</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>dynamic</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>31:0</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>stat_otf_tile_cnt</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>Tile-to-OTF accepted tile count</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>Current or last frame debug counter</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>ubwc_dec_apb_reg_blk</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>0x0074</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>APB_ADDR_STAT_OTF_LINE</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>RO</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>dynamic</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>31:0</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>stat_otf_line_cnt</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>OTF output line count</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>Current or last frame debug counter</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>ubwc_dec_apb_reg_blk</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>0x0078</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>APB_ADDR_STAT_OTF_DE</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>RO</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>dynamic</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>31:0</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>stat_otf_de_cnt</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>OTF output de &amp;&amp; ready beat count</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>Current or last frame debug counter</t>
+          <t>Read during runtime or after interrupt handling for status/debug.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I64"/>
+  <autoFilter ref="A1:I59"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3118,7 +2883,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-07 04:34:29</t>
+          <t>2026-05-14 22:08:50</t>
         </is>
       </c>
     </row>
@@ -3546,7 +3311,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>配置 CI input type、sideband、lossy、alpha mode。当前 tiled UBWC 流通常写 input_type=1。</t>
+          <t>配置 CI input type、lossy、alpha mode。当前 tiled UBWC 流通常写 input_type=1。</t>
         </is>
       </c>
     </row>
@@ -3841,7 +3606,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>DEC 自动启动</t>
+          <t>DEC 启动</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3851,7 +3616,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>硬件自动</t>
+          <t>每帧</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -3861,12 +3626,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>不需要 APB start</t>
+          <t>WRITE 0x060 bit[5]=1</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>完整地址组有效、metadata 不 busy、launch slot 可用时，硬件自动锁存本帧地址，产生 frame_start 并启动 decode。</t>
+          <t>写 START token。完整地址组和 START token 都有效，且 metadata stage 可接受新帧时，硬件锁存本帧地址并启动 decode。</t>
         </is>
       </c>
     </row>
@@ -4174,19 +3939,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Software writes metadata/tile bases for RGBA/Y and UV. A complete address set is required for each frame.</t>
+          <t>Software writes metadata/tile bases for RGBA/Y and UV. A complete address set plus a separate IRQ_CTRL[5] start write is required for each frame.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DEC auto start</t>
+          <t>DEC start token</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A decode frame starts automatically when a complete DEC address set is valid, metadata is not busy, and the metadata launch slot is free.</t>
+          <t>A decode frame starts when a complete DEC address set and a START token are both valid, metadata is not busy, and the metadata launch slot is free.</t>
         </is>
       </c>
     </row>
@@ -4234,7 +3999,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Correct IRQ is produced near the output hsync of the 4th line before frame end. Error IRQ is produced when an error condition is latched.</t>
+          <t>Correct IRQ/frame_done is produced after the final valid frame output/data completion event. Error IRQ is produced when an error condition is latched.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync register docs with APB RTL
</commit_message>
<xml_diff>
--- a/docs/ubwc_dec_reg_table.xlsx
+++ b/docs/ubwc_dec_reg_table.xlsx
@@ -2223,17 +2223,17 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>6:0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>vivo_idle_bits</t>
+          <t>vivo_idle</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Raw VIVO idle bitmap.</t>
+          <t>VIVO idle status.</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2270,17 +2270,17 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>6:0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>vivo_error_bits</t>
+          <t>vivo_error</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Raw VIVO error bitmap.</t>
+          <t>VIVO error status.</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-14 22:08:50</t>
+          <t>2026-05-19 09:33:12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update UBWC R7130 config and vectors
</commit_message>
<xml_diff>
--- a/docs/ubwc_dec_reg_table.xlsx
+++ b/docs/ubwc_dec_reg_table.xlsx
@@ -635,7 +635,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>CI input type. Software should write 1 for tiled CI.</t>
+          <t>CI input type. 1=tiled data, 0=linear data. Register reset is 0; software should write 1 for the normal tiled UBWC path.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>0x00000001</t>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>VIVO UBWC path enable.</t>
+          <t>VIVO UBWC path enable. Register reset is 0; software should write 1 before starting decode.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>meta_base_addr_rgba_y[31:0]</t>
+          <t>meta_base_addr_rgba_y_31_0</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>meta_base_addr_rgba_y[63:32]</t>
+          <t>meta_base_addr_rgba_y_63_32</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>tile_base_addr_rgba_y[31:0]</t>
+          <t>tile_base_addr_rgba_y_31_0</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>tile_base_addr_rgba_y[63:32]</t>
+          <t>tile_base_addr_rgba_y_63_32</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>meta_base_addr_uv[31:0]</t>
+          <t>meta_base_addr_uv_31_0</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>meta_base_addr_uv[63:32]</t>
+          <t>meta_base_addr_uv_63_32</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>tile_base_addr_uv[31:0]</t>
+          <t>tile_base_addr_uv_31_0</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>tile_base_addr_uv[63:32]</t>
+          <t>tile_base_addr_uv_63_32</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1793,9 +1793,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1840,9 +1840,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1887,9 +1887,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1934,9 +1934,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1981,9 +1981,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2028,9 +2028,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2075,9 +2075,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2122,9 +2122,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2169,9 +2169,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2216,9 +2216,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2263,9 +2263,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2312,7 +2312,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>0x00000001</t>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Interrupt enable.</t>
+          <t>Interrupt enable. Register reset is 0; software should write 1 when IRQ output is required.</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2404,9 +2404,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2451,9 +2451,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2498,9 +2498,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2592,9 +2592,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2639,9 +2639,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2686,9 +2686,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2733,9 +2733,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2780,9 +2780,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2827,9 +2827,9 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>dynamic</t>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-19 09:33:12</t>
+          <t>2026-05-21 13:09:24</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>使能中断。ENC IRQ_CTRL 地址为 0x060，DEC IRQ_CTRL 地址为 0x060。复位默认 irq_enable=1。</t>
+          <t>使能中断。ENC IRQ_CTRL 地址为 0x060，DEC IRQ_CTRL 地址为 0x060。寄存器复位值为 0，软件需要写 1 才使能 IRQ。</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3311,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>配置 CI input type、lossy、alpha mode。当前 tiled UBWC 流通常写 input_type=1。</t>
+          <t>配置 CI input type、lossy、alpha mode。寄存器复位值为 0，普通 tiled UBWC 路径软件应配置 ci_input_type=1。</t>
         </is>
       </c>
     </row>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>配置 vivo_ubwc_en 和 vivo_sreset。通常 vivo_ubwc_en 复位后保持 1。</t>
+          <t>配置 vivo_ubwc_en 和 vivo_sreset。寄存器复位值为 0，启动 decode 前软件应配置 vivo_ubwc_en=1。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update UBWC frame control and configuration flow
</commit_message>
<xml_diff>
--- a/docs/ubwc_dec_reg_table.xlsx
+++ b/docs/ubwc_dec_reg_table.xlsx
@@ -2883,7 +2883,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-21 13:09:24</t>
+          <t>2026-07-24 23:24:40</t>
         </is>
       </c>
     </row>
@@ -3237,7 +3237,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -3461,7 +3461,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -3493,7 +3493,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -3525,7 +3525,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -3557,7 +3557,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -3589,7 +3589,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -3621,7 +3621,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -3717,7 +3717,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>格式和尺寸不变时，tile/OTF/meta geometry 可复用；每帧只更新 base address。</t>
+          <t>格式、尺寸和输出 buffer 不变时，静态配置与唯一地址组均可持续复用。</t>
         </is>
       </c>
     </row>
@@ -3824,7 +3824,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>几何规则同 RGBA8888；只换 buffer 地址时不需要重配 geometry。</t>
+          <t>几何规则同 RGBA8888；更换 buffer 地址后重新写完整地址组并写 START。</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Y/UV 有独立 metadata/tile base；新 buffer 必须写每帧地址。</t>
+          <t>Y/UV 使用唯一一组独立 metadata/tile base；地址变化后重新写完整地址组并写 START。</t>
         </is>
       </c>
     </row>

</xml_diff>